<commit_message>
Updated substance use pathway effective levels.
</commit_message>
<xml_diff>
--- a/assets_output/04_bivariate_analysis_placements.xlsx
+++ b/assets_output/04_bivariate_analysis_placements.xlsx
@@ -863,10 +863,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1562</v>
+        <v>1660</v>
       </c>
       <c r="C30" t="n">
-        <v>24.6</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="31">
@@ -889,36 +889,36 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1164</v>
+        <v>865</v>
       </c>
       <c r="C32" t="n">
-        <v>18.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>744</v>
+        <v>854</v>
       </c>
       <c r="C33" t="n">
-        <v>11.7</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>653</v>
+        <v>744</v>
       </c>
       <c r="C34" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="35">
@@ -1019,17 +1019,17 @@
         </is>
       </c>
       <c r="B42" s="1" t="n">
-        <v>1562</v>
+        <v>1660</v>
       </c>
       <c r="C42" s="1" t="n">
-        <v>24.6</v>
+        <v>26.1</v>
       </c>
       <c r="D42" s="1" t="inlineStr"/>
       <c r="E42" t="n">
-        <v>1400</v>
+        <v>1403</v>
       </c>
       <c r="F42" t="n">
-        <v>22</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="43">
@@ -1042,10 +1042,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>86</v>
+        <v>139</v>
       </c>
       <c r="F43" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="44">
@@ -1058,10 +1058,10 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>76</v>
+        <v>118</v>
       </c>
       <c r="F44" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="45">
@@ -1111,10 +1111,10 @@
         </is>
       </c>
       <c r="B47" s="1" t="n">
-        <v>1164</v>
+        <v>865</v>
       </c>
       <c r="C47" s="1" t="n">
-        <v>18.3</v>
+        <v>13.6</v>
       </c>
       <c r="D47" s="1" t="inlineStr">
         <is>
@@ -1122,10 +1122,10 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>651</v>
+        <v>436</v>
       </c>
       <c r="F47" t="n">
-        <v>10.2</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="48">
@@ -1134,10 +1134,10 @@
       <c r="C48" s="1" t="n"/>
       <c r="D48" s="1" t="inlineStr"/>
       <c r="E48" t="n">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="F48" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="49">
@@ -1150,54 +1150,46 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>141</v>
+        <v>68</v>
       </c>
       <c r="F49" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B50" s="1" t="n">
-        <v>744</v>
+        <v>854</v>
       </c>
       <c r="C50" s="1" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="D50" s="1" t="inlineStr">
+        <v>13.4</v>
+      </c>
+      <c r="D50" s="1" t="inlineStr"/>
+      <c r="E50" t="n">
+        <v>433</v>
+      </c>
+      <c r="F50" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n"/>
+      <c r="B51" s="1" t="n"/>
+      <c r="C51" s="1" t="n"/>
+      <c r="D51" s="1" t="inlineStr">
         <is>
           <t>Unplanned</t>
         </is>
       </c>
-      <c r="E50" t="n">
-        <v>744</v>
-      </c>
-      <c r="F50" t="n">
-        <v>11.7</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="inlineStr">
-        <is>
-          <t>Internal move: backwards</t>
-        </is>
-      </c>
-      <c r="B51" s="1" t="n">
-        <v>653</v>
-      </c>
-      <c r="C51" s="1" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="D51" s="1" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>425</v>
+        <v>318</v>
       </c>
       <c r="F51" t="n">
-        <v>6.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52">
@@ -1206,30 +1198,38 @@
       <c r="C52" s="1" t="n"/>
       <c r="D52" s="1" t="inlineStr">
         <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>103</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>Returned to homelessness</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="n">
+        <v>744</v>
+      </c>
+      <c r="C53" s="1" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
           <t>Unplanned</t>
         </is>
       </c>
-      <c r="E52" t="n">
-        <v>145</v>
-      </c>
-      <c r="F52" t="n">
-        <v>2.3</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="n"/>
-      <c r="B53" s="1" t="n"/>
-      <c r="C53" s="1" t="n"/>
-      <c r="D53" s="1" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
       <c r="E53" t="n">
-        <v>83</v>
+        <v>744</v>
       </c>
       <c r="F53" t="n">
-        <v>1.3</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="54">
@@ -1481,10 +1481,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>924</v>
+        <v>1041</v>
       </c>
       <c r="C67" t="n">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D67" t="n">
         <v>88</v>
@@ -1493,10 +1493,10 @@
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="G67" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -1505,7 +1505,7 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>1562</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="68">
@@ -1549,10 +1549,10 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>705</v>
+        <v>588</v>
       </c>
       <c r="C69" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="D69" t="n">
         <v>12</v>
@@ -1561,10 +1561,10 @@
         <v>33</v>
       </c>
       <c r="F69" t="n">
-        <v>342</v>
+        <v>151</v>
       </c>
       <c r="G69" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
@@ -1573,32 +1573,32 @@
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>1164</v>
+        <v>865</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>362</v>
+        <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>70</v>
+        <v>205</v>
       </c>
       <c r="D70" t="n">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="E70" t="n">
-        <v>92</v>
+        <v>191</v>
       </c>
       <c r="F70" t="n">
-        <v>168</v>
+        <v>210</v>
       </c>
       <c r="G70" t="n">
-        <v>21</v>
+        <v>132</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
@@ -1607,32 +1607,32 @@
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>744</v>
+        <v>854</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0</v>
+        <v>362</v>
       </c>
       <c r="C71" t="n">
-        <v>218</v>
+        <v>70</v>
       </c>
       <c r="D71" t="n">
-        <v>116</v>
+        <v>31</v>
       </c>
       <c r="E71" t="n">
-        <v>191</v>
+        <v>92</v>
       </c>
       <c r="F71" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="G71" t="n">
-        <v>128</v>
+        <v>21</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
@@ -1641,7 +1641,7 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>653</v>
+        <v>744</v>
       </c>
     </row>
     <row r="72">
@@ -1873,10 +1873,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>36.4</v>
+        <v>41.1</v>
       </c>
       <c r="C81" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="D81" t="n">
         <v>20.1</v>
@@ -1885,15 +1885,15 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="G81" t="n">
-        <v>11.6</v>
+        <v>11.3</v>
       </c>
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="n">
-        <v>24.6</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="82">
@@ -1933,10 +1933,10 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>27.8</v>
+        <v>23.2</v>
       </c>
       <c r="C83" t="n">
-        <v>7.8</v>
+        <v>9.1</v>
       </c>
       <c r="D83" t="n">
         <v>2.7</v>
@@ -1945,75 +1945,75 @@
         <v>2.6</v>
       </c>
       <c r="F83" t="n">
-        <v>37</v>
+        <v>16.3</v>
       </c>
       <c r="G83" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="n">
-        <v>18.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="C84" t="n">
-        <v>8</v>
+        <v>23.4</v>
       </c>
       <c r="D84" t="n">
-        <v>7.1</v>
+        <v>26.5</v>
       </c>
       <c r="E84" t="n">
-        <v>7.3</v>
+        <v>15.1</v>
       </c>
       <c r="F84" t="n">
-        <v>18.2</v>
+        <v>22.7</v>
       </c>
       <c r="G84" t="n">
-        <v>6.6</v>
+        <v>41.5</v>
       </c>
       <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="n">
-        <v>11.7</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="C85" t="n">
-        <v>24.9</v>
+        <v>8</v>
       </c>
       <c r="D85" t="n">
-        <v>26.5</v>
+        <v>7.1</v>
       </c>
       <c r="E85" t="n">
-        <v>15.1</v>
+        <v>7.3</v>
       </c>
       <c r="F85" t="n">
-        <v>0</v>
+        <v>18.2</v>
       </c>
       <c r="G85" t="n">
-        <v>40.3</v>
+        <v>6.6</v>
       </c>
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="86">
@@ -2189,34 +2189,34 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C93" t="n">
-        <v>341</v>
+        <v>366</v>
       </c>
       <c r="D93" t="n">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="E93" t="n">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="F93" t="n">
-        <v>196</v>
+        <v>215</v>
       </c>
       <c r="G93" t="n">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="H93" t="n">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="I93" t="n">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="J93" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K93" t="n">
-        <v>1562</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="94">
@@ -2263,108 +2263,108 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C95" t="n">
-        <v>189</v>
+        <v>117</v>
       </c>
       <c r="D95" t="n">
-        <v>206</v>
+        <v>161</v>
       </c>
       <c r="E95" t="n">
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="F95" t="n">
-        <v>189</v>
+        <v>147</v>
       </c>
       <c r="G95" t="n">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="H95" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="I95" t="n">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="J95" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="K95" t="n">
-        <v>1164</v>
+        <v>865</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="C96" t="n">
-        <v>51</v>
+        <v>171</v>
       </c>
       <c r="D96" t="n">
-        <v>85</v>
+        <v>165</v>
       </c>
       <c r="E96" t="n">
+        <v>110</v>
+      </c>
+      <c r="F96" t="n">
+        <v>101</v>
+      </c>
+      <c r="G96" t="n">
+        <v>88</v>
+      </c>
+      <c r="H96" t="n">
+        <v>94</v>
+      </c>
+      <c r="I96" t="n">
         <v>72</v>
       </c>
-      <c r="F96" t="n">
-        <v>95</v>
-      </c>
-      <c r="G96" t="n">
-        <v>114</v>
-      </c>
-      <c r="H96" t="n">
-        <v>127</v>
-      </c>
-      <c r="I96" t="n">
-        <v>137</v>
-      </c>
       <c r="J96" t="n">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="K96" t="n">
-        <v>744</v>
+        <v>854</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="C97" t="n">
-        <v>124</v>
+        <v>51</v>
       </c>
       <c r="D97" t="n">
-        <v>126</v>
+        <v>85</v>
       </c>
       <c r="E97" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="F97" t="n">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="G97" t="n">
-        <v>66</v>
+        <v>114</v>
       </c>
       <c r="H97" t="n">
-        <v>73</v>
+        <v>127</v>
       </c>
       <c r="I97" t="n">
-        <v>62</v>
+        <v>137</v>
       </c>
       <c r="J97" t="n">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="K97" t="n">
-        <v>653</v>
+        <v>744</v>
       </c>
     </row>
     <row r="98">
@@ -2568,34 +2568,34 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>30.6</v>
+        <v>31.6</v>
       </c>
       <c r="C105" t="n">
-        <v>32.1</v>
+        <v>34.5</v>
       </c>
       <c r="D105" t="n">
-        <v>29</v>
+        <v>29.6</v>
       </c>
       <c r="E105" t="n">
-        <v>25.3</v>
+        <v>26.6</v>
       </c>
       <c r="F105" t="n">
-        <v>22.5</v>
+        <v>24.7</v>
       </c>
       <c r="G105" t="n">
-        <v>22</v>
+        <v>23.9</v>
       </c>
       <c r="H105" t="n">
-        <v>17.2</v>
+        <v>18.6</v>
       </c>
       <c r="I105" t="n">
-        <v>18.2</v>
+        <v>19.8</v>
       </c>
       <c r="J105" t="n">
-        <v>17.6</v>
+        <v>18</v>
       </c>
       <c r="K105" t="n">
-        <v>24.6</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="106">
@@ -2642,108 +2642,108 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>16.8</v>
+        <v>13.8</v>
       </c>
       <c r="C107" t="n">
-        <v>17.8</v>
+        <v>11</v>
       </c>
       <c r="D107" t="n">
-        <v>20</v>
+        <v>15.7</v>
       </c>
       <c r="E107" t="n">
-        <v>18.9</v>
+        <v>14.4</v>
       </c>
       <c r="F107" t="n">
-        <v>21.7</v>
+        <v>16.9</v>
       </c>
       <c r="G107" t="n">
-        <v>15.4</v>
+        <v>10.6</v>
       </c>
       <c r="H107" t="n">
-        <v>19.9</v>
+        <v>15.3</v>
       </c>
       <c r="I107" t="n">
-        <v>15.2</v>
+        <v>12</v>
       </c>
       <c r="J107" t="n">
-        <v>13.3</v>
+        <v>10.3</v>
       </c>
       <c r="K107" t="n">
-        <v>18.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>7.1</v>
+        <v>16.3</v>
       </c>
       <c r="C108" t="n">
-        <v>4.8</v>
+        <v>16.1</v>
       </c>
       <c r="D108" t="n">
-        <v>8.300000000000001</v>
+        <v>16.1</v>
       </c>
       <c r="E108" t="n">
-        <v>8</v>
+        <v>12.2</v>
       </c>
       <c r="F108" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="G108" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H108" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="I108" t="n">
         <v>10.9</v>
       </c>
-      <c r="G108" t="n">
-        <v>15.1</v>
-      </c>
-      <c r="H108" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="I108" t="n">
-        <v>20.8</v>
-      </c>
       <c r="J108" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="K108" t="n">
-        <v>11.7</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>14.3</v>
+        <v>7.1</v>
       </c>
       <c r="C109" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D109" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E109" t="n">
+        <v>8</v>
+      </c>
+      <c r="F109" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="G109" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="H109" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="I109" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="J109" t="n">
+        <v>21</v>
+      </c>
+      <c r="K109" t="n">
         <v>11.7</v>
-      </c>
-      <c r="D109" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="E109" t="n">
-        <v>9</v>
-      </c>
-      <c r="F109" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="G109" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="H109" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="I109" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="J109" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="K109" t="n">
-        <v>10.3</v>
       </c>
     </row>
     <row r="110">
@@ -2940,19 +2940,19 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="C117" t="n">
-        <v>594</v>
+        <v>657</v>
       </c>
       <c r="D117" t="n">
-        <v>412</v>
+        <v>456</v>
       </c>
       <c r="E117" t="n">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="F117" t="n">
-        <v>1562</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="118">
@@ -2984,63 +2984,63 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C119" t="n">
-        <v>354</v>
+        <v>294</v>
       </c>
       <c r="D119" t="n">
-        <v>341</v>
+        <v>300</v>
       </c>
       <c r="E119" t="n">
-        <v>346</v>
+        <v>152</v>
       </c>
       <c r="F119" t="n">
-        <v>1164</v>
+        <v>865</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>109</v>
+        <v>159</v>
       </c>
       <c r="C120" t="n">
-        <v>298</v>
+        <v>206</v>
       </c>
       <c r="D120" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E120" t="n">
-        <v>189</v>
+        <v>342</v>
       </c>
       <c r="F120" t="n">
-        <v>744</v>
+        <v>854</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>166</v>
+        <v>109</v>
       </c>
       <c r="C121" t="n">
-        <v>209</v>
+        <v>298</v>
       </c>
       <c r="D121" t="n">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E121" t="n">
-        <v>128</v>
+        <v>189</v>
       </c>
       <c r="F121" t="n">
-        <v>653</v>
+        <v>744</v>
       </c>
     </row>
     <row r="122">
@@ -3177,19 +3177,19 @@
         </is>
       </c>
       <c r="B129" t="n">
+        <v>27</v>
+      </c>
+      <c r="C129" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="D129" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="E129" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="F129" t="n">
         <v>26.1</v>
-      </c>
-      <c r="C129" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="D129" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="E129" t="n">
-        <v>20</v>
-      </c>
-      <c r="F129" t="n">
-        <v>24.6</v>
       </c>
     </row>
     <row r="130">
@@ -3221,63 +3221,63 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="C131" t="n">
-        <v>15.2</v>
+        <v>12.6</v>
       </c>
       <c r="D131" t="n">
-        <v>21.2</v>
+        <v>18.6</v>
       </c>
       <c r="E131" t="n">
-        <v>27.8</v>
+        <v>12.2</v>
       </c>
       <c r="F131" t="n">
-        <v>18.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>9.300000000000001</v>
+        <v>13.5</v>
       </c>
       <c r="C132" t="n">
-        <v>12.8</v>
+        <v>8.9</v>
       </c>
       <c r="D132" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="E132" t="n">
-        <v>15.2</v>
+        <v>27.5</v>
       </c>
       <c r="F132" t="n">
-        <v>11.7</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>14.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C133" t="n">
-        <v>9</v>
+        <v>12.8</v>
       </c>
       <c r="D133" t="n">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E133" t="n">
-        <v>10.3</v>
+        <v>15.2</v>
       </c>
       <c r="F133" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="134">
@@ -3465,10 +3465,10 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>924</v>
+        <v>1041</v>
       </c>
       <c r="C143" t="n">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D143" t="n">
         <v>88</v>
@@ -3477,10 +3477,10 @@
         <v>0</v>
       </c>
       <c r="F143" t="n">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="G143" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H143" t="n">
         <v>0</v>
@@ -3489,7 +3489,7 @@
         <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>1562</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="144">
@@ -3533,10 +3533,10 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>705</v>
+        <v>588</v>
       </c>
       <c r="C145" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="D145" t="n">
         <v>12</v>
@@ -3545,10 +3545,10 @@
         <v>33</v>
       </c>
       <c r="F145" t="n">
-        <v>342</v>
+        <v>151</v>
       </c>
       <c r="G145" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H145" t="n">
         <v>0</v>
@@ -3557,32 +3557,32 @@
         <v>0</v>
       </c>
       <c r="J145" t="n">
-        <v>1164</v>
+        <v>865</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>362</v>
+        <v>0</v>
       </c>
       <c r="C146" t="n">
-        <v>70</v>
+        <v>205</v>
       </c>
       <c r="D146" t="n">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="E146" t="n">
-        <v>92</v>
+        <v>191</v>
       </c>
       <c r="F146" t="n">
-        <v>168</v>
+        <v>210</v>
       </c>
       <c r="G146" t="n">
-        <v>21</v>
+        <v>132</v>
       </c>
       <c r="H146" t="n">
         <v>0</v>
@@ -3591,32 +3591,32 @@
         <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>744</v>
+        <v>854</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>0</v>
+        <v>362</v>
       </c>
       <c r="C147" t="n">
-        <v>218</v>
+        <v>70</v>
       </c>
       <c r="D147" t="n">
-        <v>116</v>
+        <v>31</v>
       </c>
       <c r="E147" t="n">
-        <v>191</v>
+        <v>92</v>
       </c>
       <c r="F147" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="G147" t="n">
-        <v>128</v>
+        <v>21</v>
       </c>
       <c r="H147" t="n">
         <v>0</v>
@@ -3625,7 +3625,7 @@
         <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>653</v>
+        <v>744</v>
       </c>
     </row>
     <row r="148">
@@ -3857,10 +3857,10 @@
         </is>
       </c>
       <c r="B157" t="n">
-        <v>36.4</v>
+        <v>41.1</v>
       </c>
       <c r="C157" t="n">
-        <v>34.3</v>
+        <v>34.4</v>
       </c>
       <c r="D157" t="n">
         <v>20.1</v>
@@ -3869,15 +3869,15 @@
         <v>0</v>
       </c>
       <c r="F157" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="G157" t="n">
-        <v>11.6</v>
+        <v>11.3</v>
       </c>
       <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr"/>
       <c r="J157" t="n">
-        <v>24.6</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="158">
@@ -3917,10 +3917,10 @@
         </is>
       </c>
       <c r="B159" t="n">
-        <v>27.8</v>
+        <v>23.2</v>
       </c>
       <c r="C159" t="n">
-        <v>7.8</v>
+        <v>9.1</v>
       </c>
       <c r="D159" t="n">
         <v>2.7</v>
@@ -3929,75 +3929,75 @@
         <v>2.6</v>
       </c>
       <c r="F159" t="n">
-        <v>37</v>
+        <v>16.3</v>
       </c>
       <c r="G159" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
       <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr"/>
       <c r="J159" t="n">
-        <v>18.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="C160" t="n">
-        <v>8</v>
+        <v>23.4</v>
       </c>
       <c r="D160" t="n">
-        <v>7.1</v>
+        <v>26.5</v>
       </c>
       <c r="E160" t="n">
-        <v>7.3</v>
+        <v>15.1</v>
       </c>
       <c r="F160" t="n">
-        <v>18.2</v>
+        <v>22.7</v>
       </c>
       <c r="G160" t="n">
-        <v>6.6</v>
+        <v>41.5</v>
       </c>
       <c r="H160" t="inlineStr"/>
       <c r="I160" t="inlineStr"/>
       <c r="J160" t="n">
-        <v>11.7</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="C161" t="n">
-        <v>24.9</v>
+        <v>8</v>
       </c>
       <c r="D161" t="n">
-        <v>26.5</v>
+        <v>7.1</v>
       </c>
       <c r="E161" t="n">
-        <v>15.1</v>
+        <v>7.3</v>
       </c>
       <c r="F161" t="n">
-        <v>0</v>
+        <v>18.2</v>
       </c>
       <c r="G161" t="n">
-        <v>40.3</v>
+        <v>6.6</v>
       </c>
       <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr"/>
       <c r="J161" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="162">
@@ -4273,16 +4273,16 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="C171" t="n">
-        <v>462</v>
+        <v>525</v>
       </c>
       <c r="D171" t="n">
-        <v>323</v>
+        <v>366</v>
       </c>
       <c r="E171" t="n">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="F171" t="n">
         <v>140</v>
@@ -4291,10 +4291,10 @@
         <v>84</v>
       </c>
       <c r="H171" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I171" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J171" t="n">
         <v>28</v>
@@ -4321,7 +4321,7 @@
         <v>0</v>
       </c>
       <c r="R171" t="n">
-        <v>1562</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="172">
@@ -4389,28 +4389,28 @@
         </is>
       </c>
       <c r="B173" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="C173" t="n">
-        <v>326</v>
+        <v>263</v>
       </c>
       <c r="D173" t="n">
-        <v>308</v>
+        <v>265</v>
       </c>
       <c r="E173" t="n">
-        <v>342</v>
+        <v>151</v>
       </c>
       <c r="F173" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="G173" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H173" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I173" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J173" t="n">
         <v>7</v>
@@ -4437,123 +4437,123 @@
         <v>0</v>
       </c>
       <c r="R173" t="n">
-        <v>1164</v>
+        <v>865</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="C174" t="n">
-        <v>215</v>
+        <v>0</v>
       </c>
       <c r="D174" t="n">
-        <v>115</v>
+        <v>0</v>
       </c>
       <c r="E174" t="n">
-        <v>168</v>
+        <v>210</v>
       </c>
       <c r="F174" t="n">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="G174" t="n">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="H174" t="n">
-        <v>12</v>
+        <v>71</v>
       </c>
       <c r="I174" t="n">
-        <v>21</v>
+        <v>132</v>
       </c>
       <c r="J174" t="n">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="K174" t="n">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="L174" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="M174" t="n">
         <v>0</v>
       </c>
       <c r="N174" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="O174" t="n">
-        <v>53</v>
+        <v>110</v>
       </c>
       <c r="P174" t="n">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="Q174" t="n">
         <v>0</v>
       </c>
       <c r="R174" t="n">
-        <v>744</v>
+        <v>854</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="C175" t="n">
-        <v>0</v>
+        <v>215</v>
       </c>
       <c r="D175" t="n">
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="E175" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="F175" t="n">
-        <v>89</v>
+        <v>36</v>
       </c>
       <c r="G175" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="H175" t="n">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="I175" t="n">
-        <v>128</v>
+        <v>21</v>
       </c>
       <c r="J175" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="K175" t="n">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="L175" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="M175" t="n">
         <v>0</v>
       </c>
       <c r="N175" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="O175" t="n">
-        <v>110</v>
+        <v>53</v>
       </c>
       <c r="P175" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="Q175" t="n">
         <v>0</v>
       </c>
       <c r="R175" t="n">
-        <v>653</v>
+        <v>744</v>
       </c>
     </row>
     <row r="176">
@@ -4937,16 +4937,16 @@
         </is>
       </c>
       <c r="B185" t="n">
-        <v>46.6</v>
+        <v>50.3</v>
       </c>
       <c r="C185" t="n">
-        <v>36.7</v>
+        <v>41.7</v>
       </c>
       <c r="D185" t="n">
-        <v>33.1</v>
+        <v>37.5</v>
       </c>
       <c r="E185" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="F185" t="n">
         <v>35.3</v>
@@ -4955,10 +4955,10 @@
         <v>35.6</v>
       </c>
       <c r="H185" t="n">
-        <v>31.6</v>
+        <v>32</v>
       </c>
       <c r="I185" t="n">
-        <v>11.6</v>
+        <v>11.3</v>
       </c>
       <c r="J185" t="n">
         <v>13</v>
@@ -4981,7 +4981,7 @@
       </c>
       <c r="Q185" t="inlineStr"/>
       <c r="R185" t="n">
-        <v>24.6</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="186">
@@ -5045,28 +5045,28 @@
         </is>
       </c>
       <c r="B187" t="n">
-        <v>23.8</v>
+        <v>20.1</v>
       </c>
       <c r="C187" t="n">
-        <v>25.9</v>
+        <v>20.9</v>
       </c>
       <c r="D187" t="n">
-        <v>31.5</v>
+        <v>27.1</v>
       </c>
       <c r="E187" t="n">
-        <v>37</v>
+        <v>16.3</v>
       </c>
       <c r="F187" t="n">
-        <v>9.300000000000001</v>
+        <v>11.1</v>
       </c>
       <c r="G187" t="n">
-        <v>3.4</v>
+        <v>4.7</v>
       </c>
       <c r="H187" t="n">
-        <v>9.4</v>
+        <v>10.2</v>
       </c>
       <c r="I187" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
       <c r="J187" t="n">
         <v>3.2</v>
@@ -5089,115 +5089,115 @@
       </c>
       <c r="Q187" t="inlineStr"/>
       <c r="R187" t="n">
-        <v>18.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>10.7</v>
+        <v>0</v>
       </c>
       <c r="C188" t="n">
-        <v>17.1</v>
+        <v>0</v>
       </c>
       <c r="D188" t="n">
-        <v>11.8</v>
+        <v>0</v>
       </c>
       <c r="E188" t="n">
-        <v>18.2</v>
+        <v>22.7</v>
       </c>
       <c r="F188" t="n">
-        <v>9.1</v>
+        <v>20.7</v>
       </c>
       <c r="G188" t="n">
-        <v>9.300000000000001</v>
+        <v>22</v>
       </c>
       <c r="H188" t="n">
-        <v>4.9</v>
+        <v>29.1</v>
       </c>
       <c r="I188" t="n">
-        <v>6.6</v>
+        <v>41.5</v>
       </c>
       <c r="J188" t="n">
-        <v>8.800000000000001</v>
+        <v>21.3</v>
       </c>
       <c r="K188" t="n">
-        <v>5.2</v>
+        <v>28.4</v>
       </c>
       <c r="L188" t="n">
-        <v>6.1</v>
+        <v>39.4</v>
       </c>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="n">
-        <v>8.199999999999999</v>
+        <v>11.6</v>
       </c>
       <c r="O188" t="n">
-        <v>7.9</v>
+        <v>16.3</v>
       </c>
       <c r="P188" t="n">
-        <v>5.3</v>
+        <v>15.5</v>
       </c>
       <c r="Q188" t="inlineStr"/>
       <c r="R188" t="n">
-        <v>11.7</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="C189" t="n">
-        <v>0</v>
+        <v>17.1</v>
       </c>
       <c r="D189" t="n">
-        <v>0</v>
+        <v>11.8</v>
       </c>
       <c r="E189" t="n">
-        <v>0</v>
+        <v>18.2</v>
       </c>
       <c r="F189" t="n">
-        <v>22.4</v>
+        <v>9.1</v>
       </c>
       <c r="G189" t="n">
-        <v>23.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H189" t="n">
-        <v>30.3</v>
+        <v>4.9</v>
       </c>
       <c r="I189" t="n">
-        <v>40.3</v>
+        <v>6.6</v>
       </c>
       <c r="J189" t="n">
-        <v>21.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K189" t="n">
-        <v>28.4</v>
+        <v>5.2</v>
       </c>
       <c r="L189" t="n">
-        <v>39.4</v>
+        <v>6.1</v>
       </c>
       <c r="M189" t="inlineStr"/>
       <c r="N189" t="n">
-        <v>11.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="O189" t="n">
-        <v>16.3</v>
+        <v>7.9</v>
       </c>
       <c r="P189" t="n">
-        <v>15.5</v>
+        <v>5.3</v>
       </c>
       <c r="Q189" t="inlineStr"/>
       <c r="R189" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="190">
@@ -6509,19 +6509,19 @@
         </is>
       </c>
       <c r="B249" t="n">
-        <v>481</v>
+        <v>528</v>
       </c>
       <c r="C249" t="n">
-        <v>613</v>
+        <v>653</v>
       </c>
       <c r="D249" t="n">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="E249" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F249" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G249" t="n">
         <v>20</v>
@@ -6552,7 +6552,7 @@
       <c r="S249" t="inlineStr"/>
       <c r="T249" t="inlineStr"/>
       <c r="U249" t="n">
-        <v>1562</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="250">
@@ -6621,16 +6621,16 @@
         </is>
       </c>
       <c r="B251" t="n">
-        <v>524</v>
+        <v>369</v>
       </c>
       <c r="C251" t="n">
-        <v>440</v>
+        <v>317</v>
       </c>
       <c r="D251" t="n">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="E251" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F251" t="n">
         <v>13</v>
@@ -6639,10 +6639,10 @@
         <v>13</v>
       </c>
       <c r="H251" t="n">
+        <v>1</v>
+      </c>
+      <c r="I251" t="n">
         <v>2</v>
-      </c>
-      <c r="I251" t="n">
-        <v>1</v>
       </c>
       <c r="J251" t="n">
         <v>2</v>
@@ -6662,115 +6662,115 @@
       <c r="S251" t="inlineStr"/>
       <c r="T251" t="inlineStr"/>
       <c r="U251" t="n">
-        <v>1164</v>
+        <v>865</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B252" t="n">
+        <v>289</v>
+      </c>
+      <c r="C252" t="n">
         <v>301</v>
       </c>
-      <c r="C252" t="n">
-        <v>263</v>
-      </c>
       <c r="D252" t="n">
-        <v>85</v>
+        <v>125</v>
       </c>
       <c r="E252" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="F252" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G252" t="n">
+        <v>17</v>
+      </c>
+      <c r="H252" t="n">
         <v>13</v>
-      </c>
-      <c r="H252" t="n">
-        <v>5</v>
       </c>
       <c r="I252" t="n">
         <v>7</v>
       </c>
       <c r="J252" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K252" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L252" t="n">
         <v>1</v>
       </c>
-      <c r="M252" t="inlineStr"/>
+      <c r="M252" t="n">
+        <v>2</v>
+      </c>
       <c r="N252" t="inlineStr"/>
-      <c r="O252" t="inlineStr"/>
+      <c r="O252" t="n">
+        <v>2</v>
+      </c>
       <c r="P252" t="inlineStr"/>
       <c r="Q252" t="inlineStr"/>
-      <c r="R252" t="inlineStr"/>
+      <c r="R252" t="n">
+        <v>1</v>
+      </c>
       <c r="S252" t="inlineStr"/>
       <c r="T252" t="inlineStr"/>
       <c r="U252" t="n">
-        <v>744</v>
+        <v>854</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B253" t="n">
-        <v>181</v>
+        <v>301</v>
       </c>
       <c r="C253" t="n">
-        <v>218</v>
+        <v>263</v>
       </c>
       <c r="D253" t="n">
-        <v>116</v>
+        <v>85</v>
       </c>
       <c r="E253" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="F253" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="G253" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H253" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I253" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J253" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K253" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L253" t="n">
         <v>1</v>
       </c>
-      <c r="M253" t="n">
-        <v>2</v>
-      </c>
+      <c r="M253" t="inlineStr"/>
       <c r="N253" t="inlineStr"/>
-      <c r="O253" t="n">
-        <v>2</v>
-      </c>
+      <c r="O253" t="inlineStr"/>
       <c r="P253" t="inlineStr"/>
       <c r="Q253" t="inlineStr"/>
-      <c r="R253" t="n">
-        <v>1</v>
-      </c>
+      <c r="R253" t="inlineStr"/>
       <c r="S253" t="inlineStr"/>
       <c r="T253" t="inlineStr"/>
       <c r="U253" t="n">
-        <v>653</v>
+        <v>744</v>
       </c>
     </row>
     <row r="254">
@@ -7074,19 +7074,19 @@
         </is>
       </c>
       <c r="B261" t="n">
-        <v>24.2</v>
+        <v>26.5</v>
       </c>
       <c r="C261" t="n">
-        <v>28.8</v>
+        <v>30.7</v>
       </c>
       <c r="D261" t="n">
-        <v>27.6</v>
+        <v>28.1</v>
       </c>
       <c r="E261" t="n">
-        <v>18.8</v>
+        <v>19.7</v>
       </c>
       <c r="F261" t="n">
-        <v>14.4</v>
+        <v>14.8</v>
       </c>
       <c r="G261" t="n">
         <v>10.7</v>
@@ -7117,7 +7117,7 @@
       <c r="S261" t="inlineStr"/>
       <c r="T261" t="inlineStr"/>
       <c r="U261" t="n">
-        <v>24.6</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="262">
@@ -7186,16 +7186,16 @@
         </is>
       </c>
       <c r="B263" t="n">
-        <v>26.3</v>
+        <v>18.5</v>
       </c>
       <c r="C263" t="n">
-        <v>20.7</v>
+        <v>14.9</v>
       </c>
       <c r="D263" t="n">
-        <v>11.9</v>
+        <v>10.5</v>
       </c>
       <c r="E263" t="n">
-        <v>8.300000000000001</v>
+        <v>7</v>
       </c>
       <c r="F263" t="n">
         <v>4.8</v>
@@ -7204,10 +7204,10 @@
         <v>7</v>
       </c>
       <c r="H263" t="n">
-        <v>2.3</v>
+        <v>1.1</v>
       </c>
       <c r="I263" t="n">
-        <v>1.9</v>
+        <v>3.8</v>
       </c>
       <c r="J263" t="n">
         <v>5.4</v>
@@ -7227,115 +7227,115 @@
       <c r="S263" t="inlineStr"/>
       <c r="T263" t="inlineStr"/>
       <c r="U263" t="n">
-        <v>18.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>Returned to homelessness</t>
+          <t>Internal move: backwards</t>
         </is>
       </c>
       <c r="B264" t="n">
-        <v>15.1</v>
+        <v>14.5</v>
       </c>
       <c r="C264" t="n">
-        <v>12.4</v>
+        <v>14.1</v>
       </c>
       <c r="D264" t="n">
-        <v>8.4</v>
+        <v>12.3</v>
       </c>
       <c r="E264" t="n">
-        <v>8.699999999999999</v>
+        <v>11.2</v>
       </c>
       <c r="F264" t="n">
-        <v>5.9</v>
+        <v>8.9</v>
       </c>
       <c r="G264" t="n">
-        <v>7</v>
+        <v>9.1</v>
       </c>
       <c r="H264" t="n">
-        <v>5.7</v>
+        <v>14.8</v>
       </c>
       <c r="I264" t="n">
         <v>13.5</v>
       </c>
       <c r="J264" t="n">
-        <v>13.5</v>
+        <v>21.6</v>
       </c>
       <c r="K264" t="n">
-        <v>7.7</v>
+        <v>23.1</v>
       </c>
       <c r="L264" t="n">
         <v>12.5</v>
       </c>
-      <c r="M264" t="inlineStr"/>
+      <c r="M264" t="n">
+        <v>28.6</v>
+      </c>
       <c r="N264" t="inlineStr"/>
-      <c r="O264" t="inlineStr"/>
+      <c r="O264" t="n">
+        <v>66.7</v>
+      </c>
       <c r="P264" t="inlineStr"/>
       <c r="Q264" t="inlineStr"/>
-      <c r="R264" t="inlineStr"/>
+      <c r="R264" t="n">
+        <v>100</v>
+      </c>
       <c r="S264" t="inlineStr"/>
       <c r="T264" t="inlineStr"/>
       <c r="U264" t="n">
-        <v>11.7</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>Internal move: backwards</t>
+          <t>Returned to homelessness</t>
         </is>
       </c>
       <c r="B265" t="n">
-        <v>9.1</v>
+        <v>15.1</v>
       </c>
       <c r="C265" t="n">
-        <v>10.2</v>
+        <v>12.4</v>
       </c>
       <c r="D265" t="n">
-        <v>11.4</v>
+        <v>8.4</v>
       </c>
       <c r="E265" t="n">
-        <v>10.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F265" t="n">
-        <v>9.199999999999999</v>
+        <v>5.9</v>
       </c>
       <c r="G265" t="n">
-        <v>9.1</v>
+        <v>7</v>
       </c>
       <c r="H265" t="n">
-        <v>13.6</v>
+        <v>5.7</v>
       </c>
       <c r="I265" t="n">
-        <v>15.4</v>
+        <v>13.5</v>
       </c>
       <c r="J265" t="n">
-        <v>21.6</v>
+        <v>13.5</v>
       </c>
       <c r="K265" t="n">
-        <v>23.1</v>
+        <v>7.7</v>
       </c>
       <c r="L265" t="n">
         <v>12.5</v>
       </c>
-      <c r="M265" t="n">
-        <v>28.6</v>
-      </c>
+      <c r="M265" t="inlineStr"/>
       <c r="N265" t="inlineStr"/>
-      <c r="O265" t="n">
-        <v>66.7</v>
-      </c>
+      <c r="O265" t="inlineStr"/>
       <c r="P265" t="inlineStr"/>
       <c r="Q265" t="inlineStr"/>
-      <c r="R265" t="n">
-        <v>100</v>
-      </c>
+      <c r="R265" t="inlineStr"/>
       <c r="S265" t="inlineStr"/>
       <c r="T265" t="inlineStr"/>
       <c r="U265" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="266">
@@ -7933,19 +7933,19 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>297</v>
+        <v>354</v>
       </c>
       <c r="E277" t="n">
-        <v>357</v>
+        <v>403</v>
       </c>
       <c r="F277" t="n">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="G277" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="H277" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I277" t="n">
         <v>12</v>
@@ -7990,7 +7990,7 @@
         <v>0</v>
       </c>
       <c r="W277" t="n">
-        <v>924</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="278">
@@ -8002,19 +8002,19 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>312</v>
+        <v>255</v>
       </c>
       <c r="E278" t="n">
-        <v>258</v>
+        <v>212</v>
       </c>
       <c r="F278" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="G278" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H278" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I278" t="n">
         <v>7</v>
@@ -8059,7 +8059,7 @@
         <v>0</v>
       </c>
       <c r="W278" t="n">
-        <v>705</v>
+        <v>588</v>
       </c>
     </row>
     <row r="279">
@@ -8420,19 +8420,19 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E284" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F284" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="G284" t="n">
         <v>10</v>
       </c>
       <c r="H284" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I284" t="n">
         <v>2</v>
@@ -8441,7 +8441,7 @@
         <v>2</v>
       </c>
       <c r="K284" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L284" t="n">
         <v>2</v>
@@ -8477,7 +8477,7 @@
         <v>0</v>
       </c>
       <c r="W284" t="n">
-        <v>218</v>
+        <v>205</v>
       </c>
     </row>
     <row r="285">
@@ -8489,7 +8489,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E285" t="n">
         <v>124</v>
@@ -8546,7 +8546,7 @@
         <v>0</v>
       </c>
       <c r="W285" t="n">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="286">
@@ -8558,19 +8558,19 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E286" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F286" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G286" t="n">
         <v>1</v>
       </c>
       <c r="H286" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I286" t="n">
         <v>1</v>
@@ -8579,7 +8579,7 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L286" t="n">
         <v>0</v>
@@ -8615,7 +8615,7 @@
         <v>0</v>
       </c>
       <c r="W286" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
     </row>
     <row r="287">
@@ -10090,16 +10090,16 @@
         </is>
       </c>
       <c r="D308" t="n">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="E308" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="F308" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G308" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H308" t="n">
         <v>0</v>
@@ -10108,7 +10108,7 @@
         <v>0</v>
       </c>
       <c r="J308" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K308" t="n">
         <v>0</v>
@@ -10146,7 +10146,9 @@
       <c r="V308" t="n">
         <v>0</v>
       </c>
-      <c r="W308" t="inlineStr"/>
+      <c r="W308" t="n">
+        <v>210</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="n"/>
@@ -10157,13 +10159,13 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E309" t="n">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="F309" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G309" t="n">
         <v>5</v>
@@ -10214,7 +10216,7 @@
         <v>0</v>
       </c>
       <c r="W309" t="n">
-        <v>212</v>
+        <v>193</v>
       </c>
     </row>
     <row r="310">
@@ -10226,16 +10228,16 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>166</v>
+        <v>68</v>
       </c>
       <c r="E310" t="n">
-        <v>141</v>
+        <v>61</v>
       </c>
       <c r="F310" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G310" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H310" t="n">
         <v>0</v>
@@ -10244,7 +10246,7 @@
         <v>2</v>
       </c>
       <c r="J310" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K310" t="n">
         <v>0</v>
@@ -10283,7 +10285,7 @@
         <v>0</v>
       </c>
       <c r="W310" t="n">
-        <v>342</v>
+        <v>151</v>
       </c>
     </row>
     <row r="311">
@@ -10644,10 +10646,10 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E316" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F316" t="n">
         <v>16</v>
@@ -10701,7 +10703,7 @@
         <v>0</v>
       </c>
       <c r="W316" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="317">
@@ -10716,7 +10718,7 @@
         <v>1</v>
       </c>
       <c r="E317" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F317" t="n">
         <v>7</v>
@@ -10770,7 +10772,7 @@
         <v>0</v>
       </c>
       <c r="W317" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="318">
@@ -10782,11 +10784,11 @@
         </is>
       </c>
       <c r="D318" t="n">
+        <v>0</v>
+      </c>
+      <c r="E318" t="n">
         <v>1</v>
       </c>
-      <c r="E318" t="n">
-        <v>3</v>
-      </c>
       <c r="F318" t="n">
         <v>0</v>
       </c>
@@ -10839,7 +10841,7 @@
         <v>0</v>
       </c>
       <c r="W318" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="319">
@@ -11426,19 +11428,19 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>14.9</v>
+        <v>17.8</v>
       </c>
       <c r="E329" t="n">
-        <v>16.8</v>
+        <v>18.9</v>
       </c>
       <c r="F329" t="n">
-        <v>17.3</v>
+        <v>18.1</v>
       </c>
       <c r="G329" t="n">
-        <v>8.5</v>
+        <v>9.4</v>
       </c>
       <c r="H329" t="n">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="I329" t="n">
         <v>6.4</v>
@@ -11483,7 +11485,7 @@
         <v>0</v>
       </c>
       <c r="W329" t="n">
-        <v>14.5</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="330">
@@ -11495,19 +11497,19 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>15.7</v>
+        <v>12.8</v>
       </c>
       <c r="E330" t="n">
-        <v>12.1</v>
+        <v>10</v>
       </c>
       <c r="F330" t="n">
-        <v>7.7</v>
+        <v>6.9</v>
       </c>
       <c r="G330" t="n">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="H330" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="I330" t="n">
         <v>3.7</v>
@@ -11552,7 +11554,7 @@
         <v>0</v>
       </c>
       <c r="W330" t="n">
-        <v>11.1</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="331">
@@ -11913,19 +11915,19 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="E336" t="n">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
       <c r="F336" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="G336" t="n">
         <v>1.8</v>
       </c>
       <c r="H336" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="I336" t="n">
         <v>1.1</v>
@@ -11934,7 +11936,7 @@
         <v>2.3</v>
       </c>
       <c r="K336" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="L336" t="n">
         <v>5.4</v>
@@ -11970,7 +11972,7 @@
         <v>0</v>
       </c>
       <c r="W336" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="337">
@@ -11982,7 +11984,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="E337" t="n">
         <v>5.8</v>
@@ -12039,7 +12041,7 @@
         <v>0</v>
       </c>
       <c r="W337" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="338">
@@ -12054,16 +12056,16 @@
         <v>1.8</v>
       </c>
       <c r="E338" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="F338" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="G338" t="n">
         <v>0.2</v>
       </c>
       <c r="H338" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I338" t="n">
         <v>0.5</v>
@@ -12072,7 +12074,7 @@
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="L338" t="n">
         <v>0</v>
@@ -12108,7 +12110,7 @@
         <v>0</v>
       </c>
       <c r="W338" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="339">
@@ -13583,16 +13585,16 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="E360" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F360" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="G360" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="H360" t="n">
         <v>0</v>
@@ -13601,7 +13603,7 @@
         <v>0</v>
       </c>
       <c r="J360" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="K360" t="n">
         <v>0</v>
@@ -13639,7 +13641,9 @@
       <c r="V360" t="n">
         <v>0</v>
       </c>
-      <c r="W360" t="inlineStr"/>
+      <c r="W360" t="n">
+        <v>3.3</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="1" t="n"/>
@@ -13650,13 +13654,13 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>4.6</v>
+        <v>4.1</v>
       </c>
       <c r="E361" t="n">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="F361" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="G361" t="n">
         <v>0.9</v>
@@ -13707,7 +13711,7 @@
         <v>0</v>
       </c>
       <c r="W361" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="362">
@@ -13719,16 +13723,16 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>8.300000000000001</v>
+        <v>3.4</v>
       </c>
       <c r="E362" t="n">
-        <v>6.6</v>
+        <v>2.9</v>
       </c>
       <c r="F362" t="n">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="G362" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="H362" t="n">
         <v>0</v>
@@ -13737,7 +13741,7 @@
         <v>1.1</v>
       </c>
       <c r="J362" t="n">
-        <v>2.3</v>
+        <v>1.1</v>
       </c>
       <c r="K362" t="n">
         <v>0</v>
@@ -13776,7 +13780,7 @@
         <v>0</v>
       </c>
       <c r="W362" t="n">
-        <v>5.4</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="363">
@@ -14137,10 +14141,10 @@
         </is>
       </c>
       <c r="D368" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="E368" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="F368" t="n">
         <v>1.6</v>
@@ -14194,7 +14198,7 @@
         <v>0</v>
       </c>
       <c r="W368" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="369">
@@ -14209,7 +14213,7 @@
         <v>0.1</v>
       </c>
       <c r="E369" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="F369" t="n">
         <v>0.7</v>
@@ -14275,10 +14279,10 @@
         </is>
       </c>
       <c r="D370" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E370" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F370" t="n">
         <v>0</v>
@@ -14332,7 +14336,7 @@
         <v>0</v>
       </c>
       <c r="W370" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="371">
@@ -14550,7 +14554,6 @@
     <mergeCell ref="F140:I140"/>
     <mergeCell ref="A57:A59"/>
     <mergeCell ref="B281:B288"/>
-    <mergeCell ref="C51:C53"/>
     <mergeCell ref="C57:C59"/>
     <mergeCell ref="E220:G220"/>
     <mergeCell ref="B64:E64"/>
@@ -14566,7 +14569,6 @@
     <mergeCell ref="B154:E154"/>
     <mergeCell ref="B273:B280"/>
     <mergeCell ref="F64:I64"/>
-    <mergeCell ref="B51:B53"/>
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="B365:B372"/>
     <mergeCell ref="B341:B348"/>
@@ -14576,19 +14578,21 @@
     <mergeCell ref="A357:A372"/>
     <mergeCell ref="B47:B49"/>
     <mergeCell ref="C42:C44"/>
+    <mergeCell ref="B50:B52"/>
     <mergeCell ref="A325:A356"/>
     <mergeCell ref="F168:I168"/>
     <mergeCell ref="C54:C56"/>
     <mergeCell ref="B140:E140"/>
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="A3:A8"/>
-    <mergeCell ref="A51:A53"/>
     <mergeCell ref="B333:B340"/>
     <mergeCell ref="B289:B296"/>
     <mergeCell ref="B349:B356"/>
     <mergeCell ref="A54:A56"/>
+    <mergeCell ref="A50:A52"/>
     <mergeCell ref="B42:B44"/>
     <mergeCell ref="A273:A304"/>
+    <mergeCell ref="C50:C52"/>
     <mergeCell ref="B45:B46"/>
     <mergeCell ref="J182:M182"/>
     <mergeCell ref="F154:I154"/>

</xml_diff>

<commit_message>
Fiddled with Figure 4.1
</commit_message>
<xml_diff>
--- a/assets_output/04_bivariate_analysis_placements.xlsx
+++ b/assets_output/04_bivariate_analysis_placements.xlsx
@@ -5765,7 +5765,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Table 4.16: Placement outcomes from level 3-4 by shared vs. self-contained</t>
+          <t>Table 4.16: Placement outcomes from level 3-4 by shared vs. self-contained and age categories</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6029,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Table 4.17: Placement outcomes (as column percentages) from level 3-4 by shared vs. self-contained</t>
+          <t>Table 4.17: Placement outcomes (as column percentages) from level 3-4 by shared vs. self-contained and age categories</t>
         </is>
       </c>
     </row>

</xml_diff>